<commit_message>
solved minor issues from changing timer instances and timer-channels
</commit_message>
<xml_diff>
--- a/doc/PulseZeiten.xlsx
+++ b/doc/PulseZeiten.xlsx
@@ -1,22 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29231"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\eclipse_wrk\mandelLed\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:2001_{A7E9B128-F534-47D5-B6E8-407020C844AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D00F23D-2E92-47C2-A6D6-005122DBE524}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3585" yWindow="3825" windowWidth="22410" windowHeight="15345" xr2:uid="{6C6465EA-CB0C-4969-A2CE-94929CFE4A43}"/>
+    <workbookView xWindow="-19200" yWindow="-588" windowWidth="19800" windowHeight="13548" xr2:uid="{6C6465EA-CB0C-4969-A2CE-94929CFE4A43}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -37,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="12">
   <si>
     <t>Basis</t>
   </si>
@@ -52,6 +51,27 @@
   </si>
   <si>
     <t>Aus Puls</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tim Clock </t>
+  </si>
+  <si>
+    <t>=</t>
+  </si>
+  <si>
+    <t>APB Tim Clock / Prescaler</t>
+  </si>
+  <si>
+    <t>Frequ</t>
+  </si>
+  <si>
+    <t>Tim Clock / ARR</t>
+  </si>
+  <si>
+    <t>Duty</t>
+  </si>
+  <si>
+    <t>(CCRx / ARR ) * 100</t>
   </si>
 </sst>
 </file>
@@ -423,7 +443,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{767D7DC8-A91C-4D27-82C5-9CAE008B8305}">
-  <dimension ref="D4:M10"/>
+  <dimension ref="D4:M18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="6" max="6" width="19.7109375" bestFit="1" customWidth="1"/>
@@ -626,6 +646,39 @@
         <v>0</v>
       </c>
     </row>
+    <row r="16" spans="4:13" x14ac:dyDescent="0.25">
+      <c r="D16" t="s">
+        <v>5</v>
+      </c>
+      <c r="E16" t="s">
+        <v>6</v>
+      </c>
+      <c r="F16" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="17" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D17" t="s">
+        <v>8</v>
+      </c>
+      <c r="E17" t="s">
+        <v>6</v>
+      </c>
+      <c r="F17" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="4:6" x14ac:dyDescent="0.25">
+      <c r="D18" t="s">
+        <v>10</v>
+      </c>
+      <c r="E18" t="s">
+        <v>6</v>
+      </c>
+      <c r="F18" t="s">
+        <v>11</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>